<commit_message>
Defect Register: DEF-004 (smoke usage pointed at localhost; fixed in c1514d0 on #83)
</commit_message>
<xml_diff>
--- a/docs/quality/Defect Register/Defect Register v0.1.xlsx
+++ b/docs/quality/Defect Register/Defect Register v0.1.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Defect Register" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Defect Register'!$B$10:$O$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -525,7 +525,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:O13"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="2" max="2"/>
@@ -886,8 +886,79 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="140" customHeight="1">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>DEF-004</t>
+        </is>
+      </c>
+      <c r="C14" s="4">
+        <f>DATE(2026,10,11)</f>
+        <v/>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>Review before the first smoke run</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>The smoke check's usage comment and the README directed the reader to --base-url http://localhost:&lt;port&gt;, while the server binds IPv4 loopback only (127.0.0.1, DEC-003). On Windows, Node can resolve localhost to ::1 first, so the smoke run could fail to connect.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>DEC-018 evidence item 2 (smoke check), scripts/smoke/phase0-smoke.js, README.md</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="inlineStr">
+        <is>
+          <t>S3</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t>A connection failure in the smoke run would read as a fault in the application, so the reachability evidence could be wrongly reported as failed, or time spent chasing a non-existent defect.</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t>Both smoke-check references changed to http://127.0.0.1:&lt;port&gt;. The browser guidance (README, session.js, DEC-018) is deliberately unchanged: a browser falls back from ::1 to 127.0.0.1 itself, and localhost is what makes the Secure __Host-sid cookie work over plain HTTP.</t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Commit c1514d0 (PR #83)</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="inlineStr">
+        <is>
+          <t>The corrected text in scripts/smoke/phase0-smoke.js and README.md (commit c1514d0), with the reasoning above. No automated test: the defect is in documentation, not behaviour. Not observed failing; found by review before the first run.</t>
+        </is>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>None. No release block.</t>
+        </is>
+      </c>
+      <c r="O14" s="5" t="inlineStr">
+        <is>
+          <t>Ethan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="B10:O13"/>
+  <autoFilter ref="B10:O14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>